<commit_message>
Auto update news data
</commit_message>
<xml_diff>
--- a/news_push_data/all_news/cna/20260401 中央社新聞.xlsx
+++ b/news_push_data/all_news/cna/20260401 中央社新聞.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1901,330 +1901,6 @@
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>中央社</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>NASA載人繞月任務展開倒數計時 阿提米絲2號4/1升空</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>2026/03/31 12:54</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>2026-03-31T12:54:00+08:00</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>https://www.cna.com.tw/news/aopl/202603310139.aspx</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>中央社</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>科威特油輪泊杜拜港遭伊朗攻擊 恐有漏油之虞</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>2026/03/31 12:25</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>2026-03-31T12:25:00+08:00</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>https://www.cna.com.tw/news/aopl/202603310127.aspx</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>中央社</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>美佛州州長簽署法案 棕櫚灘國際機場更名川普機場</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>2026/03/31 12:17</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>2026-03-31T12:17:00+08:00</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>https://www.cna.com.tw/news/aopl/202603310120.aspx</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>中央社</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>日本兩地配備長程飛彈 首度保有「反擊能力」</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>2026/03/31 12:09</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>2026-03-31T12:09:00+08:00</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>https://www.cna.com.tw/news/aopl/202603310115.aspx</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>中央社</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>中東戰爭第31天》川普想終戰盟邦盼續施壓 最新發展一次看</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>2026/03/31 12:05</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>2026-03-31T12:05:00+08:00</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>https://www.cna.com.tw/news/aopl/202603310112.aspx</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>中央社</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>美媒曝私下促川普續戰伊朗 波灣盟邦意向一次看</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>2026/03/31 11:54</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>2026-03-31T11:54:00+08:00</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>https://www.cna.com.tw/news/aopl/202603310104.aspx</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>中央社</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>國際能源供應不穩 李在明考慮動用緊急財政命令</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>2026/03/31 11:49</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>2026-03-31T11:49:00+08:00</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>https://www.cna.com.tw/news/aopl/202603310101.aspx</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>中央社</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>再駁美伊談判說法 伊朗：不會忘記過去教訓</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>2026/03/31 11:39</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>2026-03-31T11:39:00+08:00</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>https://www.cna.com.tw/news/aopl/202603310094.aspx</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>中央社</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>川普12度預告終戰 戰局卻陷泥淖難收場</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>2026/03/31 11:23</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>2026-03-31T11:23:00+08:00</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>https://www.cna.com.tw/news/aopl/202603310081.aspx</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>中央社</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>IMF警告：伊朗戰爭衝擊全球經濟 復甦前景轉趨黯淡</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>2026/03/31 11:19</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>2026-03-31T11:19:00+08:00</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>https://www.cna.com.tw/news/aopl/202603310077.aspx</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>中央社</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>澳洲16歲社群平台禁令 當局法遵調查恐祭重罰</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>2026/03/31 11:05</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>2026-03-31T11:05:00+08:00</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>https://www.cna.com.tw/news/aopl/202603310072.aspx</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>中央社</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>伊朗戰爭何時結束？ 尼坦雅胡：已完成過半目標</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>2026/03/31 11:01</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>2026-03-31T11:01:00+08:00</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>https://www.cna.com.tw/news/aopl/202603310070.aspx</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>